<commit_message>
feat: expose optional slab stress workflow
</commit_message>
<xml_diff>
--- a/documents_bin/calculation_book/计算书模板文件.xlsx
+++ b/documents_bin/calculation_book/计算书模板文件.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R39269ca7beef4223"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="楼板配筋" sheetId="2" r:id="R1bf815b15da244d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R7a27e97de95847dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="楼板配筋" sheetId="2" r:id="R7831546e6f4b4a3f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -183,10 +183,6 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="2">
-    <x:numFmt numFmtId="200" formatCode="0.###"/>
-    <x:numFmt numFmtId="201" formatCode="@"/>
-  </x:numFmts>
   <x:fonts count="4">
     <x:font>
       <x:sz val="11"/>
@@ -201,12 +197,12 @@
       <x:b/>
       <x:sz val="11"/>
       <x:color rgb="FFFFFFFF"/>
-      <x:name val="等线"/>
+      <x:name val="Microsoft YaHei"/>
     </x:font>
     <x:font>
       <x:sz val="10"/>
-      <x:color rgb="FF1F2937"/>
-      <x:name val="等线"/>
+      <x:color rgb="FF243B53"/>
+      <x:name val="Microsoft YaHei"/>
     </x:font>
   </x:fonts>
   <x:fills count="4">
@@ -218,66 +214,43 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF2F5D73"/>
+        <x:fgColor rgb="FF1F4E78"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFFFFF"/>
+        <x:fgColor rgb="FFF6F9FC"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
-  <x:borders count="7">
+  <x:borders count="3">
     <x:border/>
     <x:border>
       <x:left style="thin">
-        <x:color rgb="FF244958"/>
+        <x:color rgb="FFB8C4CE"/>
       </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFB8C4CE"/>
+      </x:right>
       <x:top style="thin">
-        <x:color rgb="FF244958"/>
+        <x:color rgb="FFB8C4CE"/>
       </x:top>
       <x:bottom style="thin">
-        <x:color rgb="FF244958"/>
+        <x:color rgb="FFB8C4CE"/>
       </x:bottom>
     </x:border>
     <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD7E0E8"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD7E0E8"/>
+      </x:right>
       <x:top style="thin">
-        <x:color rgb="FF244958"/>
+        <x:color rgb="FFD7E0E8"/>
       </x:top>
       <x:bottom style="thin">
-        <x:color rgb="FF244958"/>
-      </x:bottom>
-    </x:border>
-    <x:border>
-      <x:right style="thin">
-        <x:color rgb="FF244958"/>
-      </x:right>
-      <x:top style="thin">
-        <x:color rgb="FF244958"/>
-      </x:top>
-      <x:bottom style="thin">
-        <x:color rgb="FF244958"/>
-      </x:bottom>
-    </x:border>
-    <x:border>
-      <x:bottom style="thin">
-        <x:color rgb="FFD9E2E8"/>
-      </x:bottom>
-    </x:border>
-    <x:border>
-      <x:top style="thin">
-        <x:color rgb="FFD9E2E8"/>
-      </x:top>
-      <x:bottom style="thin">
-        <x:color rgb="FFD9E2E8"/>
-      </x:bottom>
-    </x:border>
-    <x:border>
-      <x:top style="thin">
-        <x:color rgb="FFD9E2E8"/>
-      </x:top>
-      <x:bottom style="thin">
-        <x:color rgb="FFAFC0CA"/>
+        <x:color rgb="FFD7E0E8"/>
       </x:bottom>
     </x:border>
   </x:borders>
@@ -286,7 +259,7 @@
       <x:alignment vertical="center"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="23">
+  <x:cellXfs count="10">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <x:alignment vertical="center"/>
     </x:xf>
@@ -299,28 +272,10 @@
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -329,32 +284,11 @@
     <x:xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="3" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="3" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="3" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="201" fontId="3" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="201" fontId="3" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="201" fontId="3" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1157,230 +1091,530 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
-      <x:c r="A1" s="9" t="str">
+      <x:c r="A1" s="5" t="str">
         <x:v>标高</x:v>
       </x:c>
-      <x:c r="B1" s="10" t="str">
+      <x:c r="B1" s="5" t="str">
         <x:v>顶层水平</x:v>
       </x:c>
-      <x:c r="C1" s="10" t="str">
+      <x:c r="C1" s="5" t="str">
         <x:v>顶层竖向</x:v>
       </x:c>
-      <x:c r="D1" s="10" t="str">
+      <x:c r="D1" s="5" t="str">
         <x:v>中层水平</x:v>
       </x:c>
-      <x:c r="E1" s="10" t="str">
+      <x:c r="E1" s="5" t="str">
         <x:v>中层竖向</x:v>
       </x:c>
-      <x:c r="F1" s="10" t="str">
+      <x:c r="F1" s="5" t="str">
         <x:v>底层水平</x:v>
       </x:c>
-      <x:c r="G1" s="10" t="str">
+      <x:c r="G1" s="5" t="str">
         <x:v>底层竖向</x:v>
       </x:c>
-      <x:c r="H1" s="11" t="str">
+      <x:c r="H1" s="5" t="str">
         <x:v>纵向拉筋</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="23" customHeight="1">
-      <x:c r="A2" s="17"/>
-      <x:c r="B2" s="20"/>
-      <x:c r="C2" s="20"/>
-      <x:c r="D2" s="20"/>
-      <x:c r="E2" s="20"/>
-      <x:c r="F2" s="20"/>
-      <x:c r="G2" s="20"/>
-      <x:c r="H2" s="20"/>
-    </x:row>
-    <x:row r="3" ht="23" customHeight="1">
-      <x:c r="A3" s="18"/>
-      <x:c r="B3" s="21"/>
-      <x:c r="C3" s="21"/>
-      <x:c r="D3" s="21"/>
-      <x:c r="E3" s="21"/>
-      <x:c r="F3" s="21"/>
-      <x:c r="G3" s="21"/>
-      <x:c r="H3" s="21"/>
-    </x:row>
-    <x:row r="4" ht="23" customHeight="1">
-      <x:c r="A4" s="18"/>
-      <x:c r="B4" s="21"/>
-      <x:c r="C4" s="21"/>
-      <x:c r="D4" s="21"/>
-      <x:c r="E4" s="21"/>
-      <x:c r="F4" s="21"/>
-      <x:c r="G4" s="21"/>
-      <x:c r="H4" s="21"/>
-    </x:row>
-    <x:row r="5" ht="23" customHeight="1">
-      <x:c r="A5" s="18"/>
-      <x:c r="B5" s="21"/>
-      <x:c r="C5" s="21"/>
-      <x:c r="D5" s="21"/>
-      <x:c r="E5" s="21"/>
-      <x:c r="F5" s="21"/>
-      <x:c r="G5" s="21"/>
-      <x:c r="H5" s="21"/>
-    </x:row>
-    <x:row r="6" ht="23" customHeight="1">
-      <x:c r="A6" s="18"/>
-      <x:c r="B6" s="21"/>
-      <x:c r="C6" s="21"/>
-      <x:c r="D6" s="21"/>
-      <x:c r="E6" s="21"/>
-      <x:c r="F6" s="21"/>
-      <x:c r="G6" s="21"/>
-      <x:c r="H6" s="21"/>
-    </x:row>
-    <x:row r="7" ht="23" customHeight="1">
-      <x:c r="A7" s="18"/>
-      <x:c r="B7" s="21"/>
-      <x:c r="C7" s="21"/>
-      <x:c r="D7" s="21"/>
-      <x:c r="E7" s="21"/>
-      <x:c r="F7" s="21"/>
-      <x:c r="G7" s="21"/>
-      <x:c r="H7" s="21"/>
-    </x:row>
-    <x:row r="8" ht="23" customHeight="1">
-      <x:c r="A8" s="18"/>
-      <x:c r="B8" s="21"/>
-      <x:c r="C8" s="21"/>
-      <x:c r="D8" s="21"/>
-      <x:c r="E8" s="21"/>
-      <x:c r="F8" s="21"/>
-      <x:c r="G8" s="21"/>
-      <x:c r="H8" s="21"/>
-    </x:row>
-    <x:row r="9" ht="23" customHeight="1">
-      <x:c r="A9" s="18"/>
-      <x:c r="B9" s="21"/>
-      <x:c r="C9" s="21"/>
-      <x:c r="D9" s="21"/>
-      <x:c r="E9" s="21"/>
-      <x:c r="F9" s="21"/>
-      <x:c r="G9" s="21"/>
-      <x:c r="H9" s="21"/>
-    </x:row>
-    <x:row r="10" ht="23" customHeight="1">
-      <x:c r="A10" s="18"/>
-      <x:c r="B10" s="21"/>
-      <x:c r="C10" s="21"/>
-      <x:c r="D10" s="21"/>
-      <x:c r="E10" s="21"/>
-      <x:c r="F10" s="21"/>
-      <x:c r="G10" s="21"/>
-      <x:c r="H10" s="21"/>
-    </x:row>
-    <x:row r="11" ht="23" customHeight="1">
-      <x:c r="A11" s="18"/>
-      <x:c r="B11" s="21"/>
-      <x:c r="C11" s="21"/>
-      <x:c r="D11" s="21"/>
-      <x:c r="E11" s="21"/>
-      <x:c r="F11" s="21"/>
-      <x:c r="G11" s="21"/>
-      <x:c r="H11" s="21"/>
-    </x:row>
-    <x:row r="12" ht="23" customHeight="1">
-      <x:c r="A12" s="18"/>
-      <x:c r="B12" s="21"/>
-      <x:c r="C12" s="21"/>
-      <x:c r="D12" s="21"/>
-      <x:c r="E12" s="21"/>
-      <x:c r="F12" s="21"/>
-      <x:c r="G12" s="21"/>
-      <x:c r="H12" s="21"/>
-    </x:row>
-    <x:row r="13" ht="23" customHeight="1">
-      <x:c r="A13" s="18"/>
-      <x:c r="B13" s="21"/>
-      <x:c r="C13" s="21"/>
-      <x:c r="D13" s="21"/>
-      <x:c r="E13" s="21"/>
-      <x:c r="F13" s="21"/>
-      <x:c r="G13" s="21"/>
-      <x:c r="H13" s="21"/>
-    </x:row>
-    <x:row r="14" ht="23" customHeight="1">
-      <x:c r="A14" s="18"/>
-      <x:c r="B14" s="21"/>
-      <x:c r="C14" s="21"/>
-      <x:c r="D14" s="21"/>
-      <x:c r="E14" s="21"/>
-      <x:c r="F14" s="21"/>
-      <x:c r="G14" s="21"/>
-      <x:c r="H14" s="21"/>
-    </x:row>
-    <x:row r="15" ht="23" customHeight="1">
-      <x:c r="A15" s="18"/>
-      <x:c r="B15" s="21"/>
-      <x:c r="C15" s="21"/>
-      <x:c r="D15" s="21"/>
-      <x:c r="E15" s="21"/>
-      <x:c r="F15" s="21"/>
-      <x:c r="G15" s="21"/>
-      <x:c r="H15" s="21"/>
-    </x:row>
-    <x:row r="16" ht="23" customHeight="1">
-      <x:c r="A16" s="18"/>
-      <x:c r="B16" s="21"/>
-      <x:c r="C16" s="21"/>
-      <x:c r="D16" s="21"/>
-      <x:c r="E16" s="21"/>
-      <x:c r="F16" s="21"/>
-      <x:c r="G16" s="21"/>
-      <x:c r="H16" s="21"/>
-    </x:row>
-    <x:row r="17" ht="23" customHeight="1">
-      <x:c r="A17" s="18"/>
-      <x:c r="B17" s="21"/>
-      <x:c r="C17" s="21"/>
-      <x:c r="D17" s="21"/>
-      <x:c r="E17" s="21"/>
-      <x:c r="F17" s="21"/>
-      <x:c r="G17" s="21"/>
-      <x:c r="H17" s="21"/>
-    </x:row>
-    <x:row r="18" ht="23" customHeight="1">
-      <x:c r="A18" s="18"/>
-      <x:c r="B18" s="21"/>
-      <x:c r="C18" s="21"/>
-      <x:c r="D18" s="21"/>
-      <x:c r="E18" s="21"/>
-      <x:c r="F18" s="21"/>
-      <x:c r="G18" s="21"/>
-      <x:c r="H18" s="21"/>
-    </x:row>
-    <x:row r="19" ht="23" customHeight="1">
-      <x:c r="A19" s="18"/>
-      <x:c r="B19" s="21"/>
-      <x:c r="C19" s="21"/>
-      <x:c r="D19" s="21"/>
-      <x:c r="E19" s="21"/>
-      <x:c r="F19" s="21"/>
-      <x:c r="G19" s="21"/>
-      <x:c r="H19" s="21"/>
-    </x:row>
-    <x:row r="20" ht="23" customHeight="1">
-      <x:c r="A20" s="18"/>
-      <x:c r="B20" s="21"/>
-      <x:c r="C20" s="21"/>
-      <x:c r="D20" s="21"/>
-      <x:c r="E20" s="21"/>
-      <x:c r="F20" s="21"/>
-      <x:c r="G20" s="21"/>
-      <x:c r="H20" s="21"/>
-    </x:row>
-    <x:row r="21" ht="23" customHeight="1">
-      <x:c r="A21" s="19"/>
-      <x:c r="B21" s="22"/>
-      <x:c r="C21" s="22"/>
-      <x:c r="D21" s="22"/>
-      <x:c r="E21" s="22"/>
-      <x:c r="F21" s="22"/>
-      <x:c r="G21" s="22"/>
-      <x:c r="H21" s="22"/>
+    <x:row r="2" ht="22" customHeight="1">
+      <x:c r="A2" s="9"/>
+      <x:c r="B2" s="9"/>
+      <x:c r="C2" s="9"/>
+      <x:c r="D2" s="9"/>
+      <x:c r="E2" s="9"/>
+      <x:c r="F2" s="9"/>
+      <x:c r="G2" s="9"/>
+      <x:c r="H2" s="9"/>
+    </x:row>
+    <x:row r="3" ht="22" customHeight="1">
+      <x:c r="A3" s="9"/>
+      <x:c r="B3" s="9"/>
+      <x:c r="C3" s="9"/>
+      <x:c r="D3" s="9"/>
+      <x:c r="E3" s="9"/>
+      <x:c r="F3" s="9"/>
+      <x:c r="G3" s="9"/>
+      <x:c r="H3" s="9"/>
+    </x:row>
+    <x:row r="4" ht="22" customHeight="1">
+      <x:c r="A4" s="9"/>
+      <x:c r="B4" s="9"/>
+      <x:c r="C4" s="9"/>
+      <x:c r="D4" s="9"/>
+      <x:c r="E4" s="9"/>
+      <x:c r="F4" s="9"/>
+      <x:c r="G4" s="9"/>
+      <x:c r="H4" s="9"/>
+    </x:row>
+    <x:row r="5" ht="22" customHeight="1">
+      <x:c r="A5" s="9"/>
+      <x:c r="B5" s="9"/>
+      <x:c r="C5" s="9"/>
+      <x:c r="D5" s="9"/>
+      <x:c r="E5" s="9"/>
+      <x:c r="F5" s="9"/>
+      <x:c r="G5" s="9"/>
+      <x:c r="H5" s="9"/>
+    </x:row>
+    <x:row r="6" ht="22" customHeight="1">
+      <x:c r="A6" s="9"/>
+      <x:c r="B6" s="9"/>
+      <x:c r="C6" s="9"/>
+      <x:c r="D6" s="9"/>
+      <x:c r="E6" s="9"/>
+      <x:c r="F6" s="9"/>
+      <x:c r="G6" s="9"/>
+      <x:c r="H6" s="9"/>
+    </x:row>
+    <x:row r="7" ht="22" customHeight="1">
+      <x:c r="A7" s="9"/>
+      <x:c r="B7" s="9"/>
+      <x:c r="C7" s="9"/>
+      <x:c r="D7" s="9"/>
+      <x:c r="E7" s="9"/>
+      <x:c r="F7" s="9"/>
+      <x:c r="G7" s="9"/>
+      <x:c r="H7" s="9"/>
+    </x:row>
+    <x:row r="8" ht="22" customHeight="1">
+      <x:c r="A8" s="9"/>
+      <x:c r="B8" s="9"/>
+      <x:c r="C8" s="9"/>
+      <x:c r="D8" s="9"/>
+      <x:c r="E8" s="9"/>
+      <x:c r="F8" s="9"/>
+      <x:c r="G8" s="9"/>
+      <x:c r="H8" s="9"/>
+    </x:row>
+    <x:row r="9" ht="22" customHeight="1">
+      <x:c r="A9" s="9"/>
+      <x:c r="B9" s="9"/>
+      <x:c r="C9" s="9"/>
+      <x:c r="D9" s="9"/>
+      <x:c r="E9" s="9"/>
+      <x:c r="F9" s="9"/>
+      <x:c r="G9" s="9"/>
+      <x:c r="H9" s="9"/>
+    </x:row>
+    <x:row r="10" ht="22" customHeight="1">
+      <x:c r="A10" s="9"/>
+      <x:c r="B10" s="9"/>
+      <x:c r="C10" s="9"/>
+      <x:c r="D10" s="9"/>
+      <x:c r="E10" s="9"/>
+      <x:c r="F10" s="9"/>
+      <x:c r="G10" s="9"/>
+      <x:c r="H10" s="9"/>
+    </x:row>
+    <x:row r="11" ht="22" customHeight="1">
+      <x:c r="A11" s="9"/>
+      <x:c r="B11" s="9"/>
+      <x:c r="C11" s="9"/>
+      <x:c r="D11" s="9"/>
+      <x:c r="E11" s="9"/>
+      <x:c r="F11" s="9"/>
+      <x:c r="G11" s="9"/>
+      <x:c r="H11" s="9"/>
+    </x:row>
+    <x:row r="12" ht="22" customHeight="1">
+      <x:c r="A12" s="9"/>
+      <x:c r="B12" s="9"/>
+      <x:c r="C12" s="9"/>
+      <x:c r="D12" s="9"/>
+      <x:c r="E12" s="9"/>
+      <x:c r="F12" s="9"/>
+      <x:c r="G12" s="9"/>
+      <x:c r="H12" s="9"/>
+    </x:row>
+    <x:row r="13" ht="22" customHeight="1">
+      <x:c r="A13" s="9"/>
+      <x:c r="B13" s="9"/>
+      <x:c r="C13" s="9"/>
+      <x:c r="D13" s="9"/>
+      <x:c r="E13" s="9"/>
+      <x:c r="F13" s="9"/>
+      <x:c r="G13" s="9"/>
+      <x:c r="H13" s="9"/>
+    </x:row>
+    <x:row r="14" ht="22" customHeight="1">
+      <x:c r="A14" s="9"/>
+      <x:c r="B14" s="9"/>
+      <x:c r="C14" s="9"/>
+      <x:c r="D14" s="9"/>
+      <x:c r="E14" s="9"/>
+      <x:c r="F14" s="9"/>
+      <x:c r="G14" s="9"/>
+      <x:c r="H14" s="9"/>
+    </x:row>
+    <x:row r="15" ht="22" customHeight="1">
+      <x:c r="A15" s="9"/>
+      <x:c r="B15" s="9"/>
+      <x:c r="C15" s="9"/>
+      <x:c r="D15" s="9"/>
+      <x:c r="E15" s="9"/>
+      <x:c r="F15" s="9"/>
+      <x:c r="G15" s="9"/>
+      <x:c r="H15" s="9"/>
+    </x:row>
+    <x:row r="16" ht="22" customHeight="1">
+      <x:c r="A16" s="9"/>
+      <x:c r="B16" s="9"/>
+      <x:c r="C16" s="9"/>
+      <x:c r="D16" s="9"/>
+      <x:c r="E16" s="9"/>
+      <x:c r="F16" s="9"/>
+      <x:c r="G16" s="9"/>
+      <x:c r="H16" s="9"/>
+    </x:row>
+    <x:row r="17" ht="22" customHeight="1">
+      <x:c r="A17" s="9"/>
+      <x:c r="B17" s="9"/>
+      <x:c r="C17" s="9"/>
+      <x:c r="D17" s="9"/>
+      <x:c r="E17" s="9"/>
+      <x:c r="F17" s="9"/>
+      <x:c r="G17" s="9"/>
+      <x:c r="H17" s="9"/>
+    </x:row>
+    <x:row r="18" ht="22" customHeight="1">
+      <x:c r="A18" s="9"/>
+      <x:c r="B18" s="9"/>
+      <x:c r="C18" s="9"/>
+      <x:c r="D18" s="9"/>
+      <x:c r="E18" s="9"/>
+      <x:c r="F18" s="9"/>
+      <x:c r="G18" s="9"/>
+      <x:c r="H18" s="9"/>
+    </x:row>
+    <x:row r="19" ht="22" customHeight="1">
+      <x:c r="A19" s="9"/>
+      <x:c r="B19" s="9"/>
+      <x:c r="C19" s="9"/>
+      <x:c r="D19" s="9"/>
+      <x:c r="E19" s="9"/>
+      <x:c r="F19" s="9"/>
+      <x:c r="G19" s="9"/>
+      <x:c r="H19" s="9"/>
+    </x:row>
+    <x:row r="20" ht="22" customHeight="1">
+      <x:c r="A20" s="9"/>
+      <x:c r="B20" s="9"/>
+      <x:c r="C20" s="9"/>
+      <x:c r="D20" s="9"/>
+      <x:c r="E20" s="9"/>
+      <x:c r="F20" s="9"/>
+      <x:c r="G20" s="9"/>
+      <x:c r="H20" s="9"/>
+    </x:row>
+    <x:row r="21" ht="22" customHeight="1">
+      <x:c r="A21" s="9"/>
+      <x:c r="B21" s="9"/>
+      <x:c r="C21" s="9"/>
+      <x:c r="D21" s="9"/>
+      <x:c r="E21" s="9"/>
+      <x:c r="F21" s="9"/>
+      <x:c r="G21" s="9"/>
+      <x:c r="H21" s="9"/>
+    </x:row>
+    <x:row r="22" ht="22" customHeight="1">
+      <x:c r="A22" s="9"/>
+      <x:c r="B22" s="9"/>
+      <x:c r="C22" s="9"/>
+      <x:c r="D22" s="9"/>
+      <x:c r="E22" s="9"/>
+      <x:c r="F22" s="9"/>
+      <x:c r="G22" s="9"/>
+      <x:c r="H22" s="9"/>
+    </x:row>
+    <x:row r="23" ht="22" customHeight="1">
+      <x:c r="A23" s="9"/>
+      <x:c r="B23" s="9"/>
+      <x:c r="C23" s="9"/>
+      <x:c r="D23" s="9"/>
+      <x:c r="E23" s="9"/>
+      <x:c r="F23" s="9"/>
+      <x:c r="G23" s="9"/>
+      <x:c r="H23" s="9"/>
+    </x:row>
+    <x:row r="24" ht="22" customHeight="1">
+      <x:c r="A24" s="9"/>
+      <x:c r="B24" s="9"/>
+      <x:c r="C24" s="9"/>
+      <x:c r="D24" s="9"/>
+      <x:c r="E24" s="9"/>
+      <x:c r="F24" s="9"/>
+      <x:c r="G24" s="9"/>
+      <x:c r="H24" s="9"/>
+    </x:row>
+    <x:row r="25" ht="22" customHeight="1">
+      <x:c r="A25" s="9"/>
+      <x:c r="B25" s="9"/>
+      <x:c r="C25" s="9"/>
+      <x:c r="D25" s="9"/>
+      <x:c r="E25" s="9"/>
+      <x:c r="F25" s="9"/>
+      <x:c r="G25" s="9"/>
+      <x:c r="H25" s="9"/>
+    </x:row>
+    <x:row r="26" ht="22" customHeight="1">
+      <x:c r="A26" s="9"/>
+      <x:c r="B26" s="9"/>
+      <x:c r="C26" s="9"/>
+      <x:c r="D26" s="9"/>
+      <x:c r="E26" s="9"/>
+      <x:c r="F26" s="9"/>
+      <x:c r="G26" s="9"/>
+      <x:c r="H26" s="9"/>
+    </x:row>
+    <x:row r="27" ht="22" customHeight="1">
+      <x:c r="A27" s="9"/>
+      <x:c r="B27" s="9"/>
+      <x:c r="C27" s="9"/>
+      <x:c r="D27" s="9"/>
+      <x:c r="E27" s="9"/>
+      <x:c r="F27" s="9"/>
+      <x:c r="G27" s="9"/>
+      <x:c r="H27" s="9"/>
+    </x:row>
+    <x:row r="28" ht="22" customHeight="1">
+      <x:c r="A28" s="9"/>
+      <x:c r="B28" s="9"/>
+      <x:c r="C28" s="9"/>
+      <x:c r="D28" s="9"/>
+      <x:c r="E28" s="9"/>
+      <x:c r="F28" s="9"/>
+      <x:c r="G28" s="9"/>
+      <x:c r="H28" s="9"/>
+    </x:row>
+    <x:row r="29" ht="22" customHeight="1">
+      <x:c r="A29" s="9"/>
+      <x:c r="B29" s="9"/>
+      <x:c r="C29" s="9"/>
+      <x:c r="D29" s="9"/>
+      <x:c r="E29" s="9"/>
+      <x:c r="F29" s="9"/>
+      <x:c r="G29" s="9"/>
+      <x:c r="H29" s="9"/>
+    </x:row>
+    <x:row r="30" ht="22" customHeight="1">
+      <x:c r="A30" s="9"/>
+      <x:c r="B30" s="9"/>
+      <x:c r="C30" s="9"/>
+      <x:c r="D30" s="9"/>
+      <x:c r="E30" s="9"/>
+      <x:c r="F30" s="9"/>
+      <x:c r="G30" s="9"/>
+      <x:c r="H30" s="9"/>
+    </x:row>
+    <x:row r="31" ht="22" customHeight="1">
+      <x:c r="A31" s="9"/>
+      <x:c r="B31" s="9"/>
+      <x:c r="C31" s="9"/>
+      <x:c r="D31" s="9"/>
+      <x:c r="E31" s="9"/>
+      <x:c r="F31" s="9"/>
+      <x:c r="G31" s="9"/>
+      <x:c r="H31" s="9"/>
+    </x:row>
+    <x:row r="32" ht="22" customHeight="1">
+      <x:c r="A32" s="9"/>
+      <x:c r="B32" s="9"/>
+      <x:c r="C32" s="9"/>
+      <x:c r="D32" s="9"/>
+      <x:c r="E32" s="9"/>
+      <x:c r="F32" s="9"/>
+      <x:c r="G32" s="9"/>
+      <x:c r="H32" s="9"/>
+    </x:row>
+    <x:row r="33" ht="22" customHeight="1">
+      <x:c r="A33" s="9"/>
+      <x:c r="B33" s="9"/>
+      <x:c r="C33" s="9"/>
+      <x:c r="D33" s="9"/>
+      <x:c r="E33" s="9"/>
+      <x:c r="F33" s="9"/>
+      <x:c r="G33" s="9"/>
+      <x:c r="H33" s="9"/>
+    </x:row>
+    <x:row r="34" ht="22" customHeight="1">
+      <x:c r="A34" s="9"/>
+      <x:c r="B34" s="9"/>
+      <x:c r="C34" s="9"/>
+      <x:c r="D34" s="9"/>
+      <x:c r="E34" s="9"/>
+      <x:c r="F34" s="9"/>
+      <x:c r="G34" s="9"/>
+      <x:c r="H34" s="9"/>
+    </x:row>
+    <x:row r="35" ht="22" customHeight="1">
+      <x:c r="A35" s="9"/>
+      <x:c r="B35" s="9"/>
+      <x:c r="C35" s="9"/>
+      <x:c r="D35" s="9"/>
+      <x:c r="E35" s="9"/>
+      <x:c r="F35" s="9"/>
+      <x:c r="G35" s="9"/>
+      <x:c r="H35" s="9"/>
+    </x:row>
+    <x:row r="36" ht="22" customHeight="1">
+      <x:c r="A36" s="9"/>
+      <x:c r="B36" s="9"/>
+      <x:c r="C36" s="9"/>
+      <x:c r="D36" s="9"/>
+      <x:c r="E36" s="9"/>
+      <x:c r="F36" s="9"/>
+      <x:c r="G36" s="9"/>
+      <x:c r="H36" s="9"/>
+    </x:row>
+    <x:row r="37" ht="22" customHeight="1">
+      <x:c r="A37" s="9"/>
+      <x:c r="B37" s="9"/>
+      <x:c r="C37" s="9"/>
+      <x:c r="D37" s="9"/>
+      <x:c r="E37" s="9"/>
+      <x:c r="F37" s="9"/>
+      <x:c r="G37" s="9"/>
+      <x:c r="H37" s="9"/>
+    </x:row>
+    <x:row r="38" ht="22" customHeight="1">
+      <x:c r="A38" s="9"/>
+      <x:c r="B38" s="9"/>
+      <x:c r="C38" s="9"/>
+      <x:c r="D38" s="9"/>
+      <x:c r="E38" s="9"/>
+      <x:c r="F38" s="9"/>
+      <x:c r="G38" s="9"/>
+      <x:c r="H38" s="9"/>
+    </x:row>
+    <x:row r="39" ht="22" customHeight="1">
+      <x:c r="A39" s="9"/>
+      <x:c r="B39" s="9"/>
+      <x:c r="C39" s="9"/>
+      <x:c r="D39" s="9"/>
+      <x:c r="E39" s="9"/>
+      <x:c r="F39" s="9"/>
+      <x:c r="G39" s="9"/>
+      <x:c r="H39" s="9"/>
+    </x:row>
+    <x:row r="40" ht="22" customHeight="1">
+      <x:c r="A40" s="9"/>
+      <x:c r="B40" s="9"/>
+      <x:c r="C40" s="9"/>
+      <x:c r="D40" s="9"/>
+      <x:c r="E40" s="9"/>
+      <x:c r="F40" s="9"/>
+      <x:c r="G40" s="9"/>
+      <x:c r="H40" s="9"/>
+    </x:row>
+    <x:row r="41" ht="22" customHeight="1">
+      <x:c r="A41" s="9"/>
+      <x:c r="B41" s="9"/>
+      <x:c r="C41" s="9"/>
+      <x:c r="D41" s="9"/>
+      <x:c r="E41" s="9"/>
+      <x:c r="F41" s="9"/>
+      <x:c r="G41" s="9"/>
+      <x:c r="H41" s="9"/>
+    </x:row>
+    <x:row r="42" ht="22" customHeight="1">
+      <x:c r="A42" s="9"/>
+      <x:c r="B42" s="9"/>
+      <x:c r="C42" s="9"/>
+      <x:c r="D42" s="9"/>
+      <x:c r="E42" s="9"/>
+      <x:c r="F42" s="9"/>
+      <x:c r="G42" s="9"/>
+      <x:c r="H42" s="9"/>
+    </x:row>
+    <x:row r="43" ht="22" customHeight="1">
+      <x:c r="A43" s="9"/>
+      <x:c r="B43" s="9"/>
+      <x:c r="C43" s="9"/>
+      <x:c r="D43" s="9"/>
+      <x:c r="E43" s="9"/>
+      <x:c r="F43" s="9"/>
+      <x:c r="G43" s="9"/>
+      <x:c r="H43" s="9"/>
+    </x:row>
+    <x:row r="44" ht="22" customHeight="1">
+      <x:c r="A44" s="9"/>
+      <x:c r="B44" s="9"/>
+      <x:c r="C44" s="9"/>
+      <x:c r="D44" s="9"/>
+      <x:c r="E44" s="9"/>
+      <x:c r="F44" s="9"/>
+      <x:c r="G44" s="9"/>
+      <x:c r="H44" s="9"/>
+    </x:row>
+    <x:row r="45" ht="22" customHeight="1">
+      <x:c r="A45" s="9"/>
+      <x:c r="B45" s="9"/>
+      <x:c r="C45" s="9"/>
+      <x:c r="D45" s="9"/>
+      <x:c r="E45" s="9"/>
+      <x:c r="F45" s="9"/>
+      <x:c r="G45" s="9"/>
+      <x:c r="H45" s="9"/>
+    </x:row>
+    <x:row r="46" ht="22" customHeight="1">
+      <x:c r="A46" s="9"/>
+      <x:c r="B46" s="9"/>
+      <x:c r="C46" s="9"/>
+      <x:c r="D46" s="9"/>
+      <x:c r="E46" s="9"/>
+      <x:c r="F46" s="9"/>
+      <x:c r="G46" s="9"/>
+      <x:c r="H46" s="9"/>
+    </x:row>
+    <x:row r="47" ht="22" customHeight="1">
+      <x:c r="A47" s="9"/>
+      <x:c r="B47" s="9"/>
+      <x:c r="C47" s="9"/>
+      <x:c r="D47" s="9"/>
+      <x:c r="E47" s="9"/>
+      <x:c r="F47" s="9"/>
+      <x:c r="G47" s="9"/>
+      <x:c r="H47" s="9"/>
+    </x:row>
+    <x:row r="48" ht="22" customHeight="1">
+      <x:c r="A48" s="9"/>
+      <x:c r="B48" s="9"/>
+      <x:c r="C48" s="9"/>
+      <x:c r="D48" s="9"/>
+      <x:c r="E48" s="9"/>
+      <x:c r="F48" s="9"/>
+      <x:c r="G48" s="9"/>
+      <x:c r="H48" s="9"/>
+    </x:row>
+    <x:row r="49" ht="22" customHeight="1">
+      <x:c r="A49" s="9"/>
+      <x:c r="B49" s="9"/>
+      <x:c r="C49" s="9"/>
+      <x:c r="D49" s="9"/>
+      <x:c r="E49" s="9"/>
+      <x:c r="F49" s="9"/>
+      <x:c r="G49" s="9"/>
+      <x:c r="H49" s="9"/>
+    </x:row>
+    <x:row r="50" ht="22" customHeight="1">
+      <x:c r="A50" s="9"/>
+      <x:c r="B50" s="9"/>
+      <x:c r="C50" s="9"/>
+      <x:c r="D50" s="9"/>
+      <x:c r="E50" s="9"/>
+      <x:c r="F50" s="9"/>
+      <x:c r="G50" s="9"/>
+      <x:c r="H50" s="9"/>
+    </x:row>
+    <x:row r="51" ht="22" customHeight="1">
+      <x:c r="A51" s="9"/>
+      <x:c r="B51" s="9"/>
+      <x:c r="C51" s="9"/>
+      <x:c r="D51" s="9"/>
+      <x:c r="E51" s="9"/>
+      <x:c r="F51" s="9"/>
+      <x:c r="G51" s="9"/>
+      <x:c r="H51" s="9"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
chore: update calculation book templates
</commit_message>
<xml_diff>
--- a/documents_bin/calculation_book/计算书模板文件.xlsx
+++ b/documents_bin/calculation_book/计算书模板文件.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R7a27e97de95847dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="楼板配筋" sheetId="2" r:id="R7831546e6f4b4a3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rc5bddfa0dea5494e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="楼板配筋" sheetId="2" r:id="Reb2aa92fbd2241eb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -183,6 +183,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:numFmts count="1">
+    <x:numFmt numFmtId="200" formatCode="0.00&quot;m&quot;"/>
+  </x:numFmts>
   <x:fonts count="4">
     <x:font>
       <x:sz val="11"/>
@@ -197,15 +200,15 @@
       <x:b/>
       <x:sz val="11"/>
       <x:color rgb="FFFFFFFF"/>
-      <x:name val="Microsoft YaHei"/>
+      <x:name val="等线"/>
     </x:font>
     <x:font>
-      <x:sz val="10"/>
-      <x:color rgb="FF243B53"/>
-      <x:name val="Microsoft YaHei"/>
+      <x:sz val="11"/>
+      <x:color rgb="FF1F2937"/>
+      <x:name val="等线"/>
     </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="5">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -219,38 +222,29 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFF6F9FC"/>
+        <x:fgColor rgb="FFF7FAFC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEEF2F6"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
-  <x:borders count="3">
+  <x:borders count="2">
     <x:border/>
     <x:border>
       <x:left style="thin">
-        <x:color rgb="FFB8C4CE"/>
+        <x:color rgb="FFB8C5D1"/>
       </x:left>
       <x:right style="thin">
-        <x:color rgb="FFB8C4CE"/>
+        <x:color rgb="FFB8C5D1"/>
       </x:right>
       <x:top style="thin">
-        <x:color rgb="FFB8C4CE"/>
+        <x:color rgb="FFB8C5D1"/>
       </x:top>
       <x:bottom style="thin">
-        <x:color rgb="FFB8C4CE"/>
-      </x:bottom>
-    </x:border>
-    <x:border>
-      <x:left style="thin">
-        <x:color rgb="FFD7E0E8"/>
-      </x:left>
-      <x:right style="thin">
-        <x:color rgb="FFD7E0E8"/>
-      </x:right>
-      <x:top style="thin">
-        <x:color rgb="FFD7E0E8"/>
-      </x:top>
-      <x:bottom style="thin">
-        <x:color rgb="FFD7E0E8"/>
+        <x:color rgb="FFB8C5D1"/>
       </x:bottom>
     </x:border>
   </x:borders>
@@ -263,32 +257,32 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
+    <x:xf numFmtId="200" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1080,14 +1074,14 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="19" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
@@ -1116,505 +1110,27 @@
         <x:v>纵向拉筋</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="22" customHeight="1">
-      <x:c r="A2" s="9"/>
-      <x:c r="B2" s="9"/>
-      <x:c r="C2" s="9"/>
-      <x:c r="D2" s="9"/>
-      <x:c r="E2" s="9"/>
-      <x:c r="F2" s="9"/>
-      <x:c r="G2" s="9"/>
-      <x:c r="H2" s="9"/>
-    </x:row>
-    <x:row r="3" ht="22" customHeight="1">
-      <x:c r="A3" s="9"/>
-      <x:c r="B3" s="9"/>
-      <x:c r="C3" s="9"/>
-      <x:c r="D3" s="9"/>
-      <x:c r="E3" s="9"/>
-      <x:c r="F3" s="9"/>
-      <x:c r="G3" s="9"/>
-      <x:c r="H3" s="9"/>
-    </x:row>
-    <x:row r="4" ht="22" customHeight="1">
-      <x:c r="A4" s="9"/>
-      <x:c r="B4" s="9"/>
-      <x:c r="C4" s="9"/>
-      <x:c r="D4" s="9"/>
-      <x:c r="E4" s="9"/>
-      <x:c r="F4" s="9"/>
-      <x:c r="G4" s="9"/>
-      <x:c r="H4" s="9"/>
-    </x:row>
-    <x:row r="5" ht="22" customHeight="1">
-      <x:c r="A5" s="9"/>
-      <x:c r="B5" s="9"/>
-      <x:c r="C5" s="9"/>
-      <x:c r="D5" s="9"/>
-      <x:c r="E5" s="9"/>
-      <x:c r="F5" s="9"/>
-      <x:c r="G5" s="9"/>
-      <x:c r="H5" s="9"/>
-    </x:row>
-    <x:row r="6" ht="22" customHeight="1">
-      <x:c r="A6" s="9"/>
-      <x:c r="B6" s="9"/>
-      <x:c r="C6" s="9"/>
-      <x:c r="D6" s="9"/>
-      <x:c r="E6" s="9"/>
-      <x:c r="F6" s="9"/>
-      <x:c r="G6" s="9"/>
-      <x:c r="H6" s="9"/>
-    </x:row>
-    <x:row r="7" ht="22" customHeight="1">
-      <x:c r="A7" s="9"/>
-      <x:c r="B7" s="9"/>
-      <x:c r="C7" s="9"/>
-      <x:c r="D7" s="9"/>
-      <x:c r="E7" s="9"/>
-      <x:c r="F7" s="9"/>
-      <x:c r="G7" s="9"/>
-      <x:c r="H7" s="9"/>
-    </x:row>
-    <x:row r="8" ht="22" customHeight="1">
-      <x:c r="A8" s="9"/>
-      <x:c r="B8" s="9"/>
-      <x:c r="C8" s="9"/>
-      <x:c r="D8" s="9"/>
-      <x:c r="E8" s="9"/>
-      <x:c r="F8" s="9"/>
-      <x:c r="G8" s="9"/>
-      <x:c r="H8" s="9"/>
-    </x:row>
-    <x:row r="9" ht="22" customHeight="1">
-      <x:c r="A9" s="9"/>
-      <x:c r="B9" s="9"/>
-      <x:c r="C9" s="9"/>
-      <x:c r="D9" s="9"/>
-      <x:c r="E9" s="9"/>
-      <x:c r="F9" s="9"/>
-      <x:c r="G9" s="9"/>
-      <x:c r="H9" s="9"/>
-    </x:row>
-    <x:row r="10" ht="22" customHeight="1">
-      <x:c r="A10" s="9"/>
-      <x:c r="B10" s="9"/>
-      <x:c r="C10" s="9"/>
-      <x:c r="D10" s="9"/>
-      <x:c r="E10" s="9"/>
-      <x:c r="F10" s="9"/>
-      <x:c r="G10" s="9"/>
-      <x:c r="H10" s="9"/>
-    </x:row>
-    <x:row r="11" ht="22" customHeight="1">
-      <x:c r="A11" s="9"/>
-      <x:c r="B11" s="9"/>
-      <x:c r="C11" s="9"/>
-      <x:c r="D11" s="9"/>
-      <x:c r="E11" s="9"/>
-      <x:c r="F11" s="9"/>
-      <x:c r="G11" s="9"/>
-      <x:c r="H11" s="9"/>
-    </x:row>
-    <x:row r="12" ht="22" customHeight="1">
-      <x:c r="A12" s="9"/>
-      <x:c r="B12" s="9"/>
-      <x:c r="C12" s="9"/>
-      <x:c r="D12" s="9"/>
-      <x:c r="E12" s="9"/>
-      <x:c r="F12" s="9"/>
-      <x:c r="G12" s="9"/>
-      <x:c r="H12" s="9"/>
-    </x:row>
-    <x:row r="13" ht="22" customHeight="1">
-      <x:c r="A13" s="9"/>
-      <x:c r="B13" s="9"/>
-      <x:c r="C13" s="9"/>
-      <x:c r="D13" s="9"/>
-      <x:c r="E13" s="9"/>
-      <x:c r="F13" s="9"/>
-      <x:c r="G13" s="9"/>
-      <x:c r="H13" s="9"/>
-    </x:row>
-    <x:row r="14" ht="22" customHeight="1">
-      <x:c r="A14" s="9"/>
-      <x:c r="B14" s="9"/>
-      <x:c r="C14" s="9"/>
-      <x:c r="D14" s="9"/>
-      <x:c r="E14" s="9"/>
-      <x:c r="F14" s="9"/>
-      <x:c r="G14" s="9"/>
-      <x:c r="H14" s="9"/>
-    </x:row>
-    <x:row r="15" ht="22" customHeight="1">
-      <x:c r="A15" s="9"/>
-      <x:c r="B15" s="9"/>
-      <x:c r="C15" s="9"/>
-      <x:c r="D15" s="9"/>
-      <x:c r="E15" s="9"/>
-      <x:c r="F15" s="9"/>
-      <x:c r="G15" s="9"/>
-      <x:c r="H15" s="9"/>
-    </x:row>
-    <x:row r="16" ht="22" customHeight="1">
-      <x:c r="A16" s="9"/>
-      <x:c r="B16" s="9"/>
-      <x:c r="C16" s="9"/>
-      <x:c r="D16" s="9"/>
-      <x:c r="E16" s="9"/>
-      <x:c r="F16" s="9"/>
-      <x:c r="G16" s="9"/>
-      <x:c r="H16" s="9"/>
-    </x:row>
-    <x:row r="17" ht="22" customHeight="1">
-      <x:c r="A17" s="9"/>
-      <x:c r="B17" s="9"/>
-      <x:c r="C17" s="9"/>
-      <x:c r="D17" s="9"/>
-      <x:c r="E17" s="9"/>
-      <x:c r="F17" s="9"/>
-      <x:c r="G17" s="9"/>
-      <x:c r="H17" s="9"/>
-    </x:row>
-    <x:row r="18" ht="22" customHeight="1">
-      <x:c r="A18" s="9"/>
-      <x:c r="B18" s="9"/>
-      <x:c r="C18" s="9"/>
-      <x:c r="D18" s="9"/>
-      <x:c r="E18" s="9"/>
-      <x:c r="F18" s="9"/>
-      <x:c r="G18" s="9"/>
-      <x:c r="H18" s="9"/>
-    </x:row>
-    <x:row r="19" ht="22" customHeight="1">
-      <x:c r="A19" s="9"/>
-      <x:c r="B19" s="9"/>
-      <x:c r="C19" s="9"/>
-      <x:c r="D19" s="9"/>
-      <x:c r="E19" s="9"/>
-      <x:c r="F19" s="9"/>
-      <x:c r="G19" s="9"/>
-      <x:c r="H19" s="9"/>
-    </x:row>
-    <x:row r="20" ht="22" customHeight="1">
-      <x:c r="A20" s="9"/>
-      <x:c r="B20" s="9"/>
-      <x:c r="C20" s="9"/>
-      <x:c r="D20" s="9"/>
-      <x:c r="E20" s="9"/>
-      <x:c r="F20" s="9"/>
-      <x:c r="G20" s="9"/>
-      <x:c r="H20" s="9"/>
-    </x:row>
-    <x:row r="21" ht="22" customHeight="1">
-      <x:c r="A21" s="9"/>
-      <x:c r="B21" s="9"/>
-      <x:c r="C21" s="9"/>
-      <x:c r="D21" s="9"/>
-      <x:c r="E21" s="9"/>
-      <x:c r="F21" s="9"/>
-      <x:c r="G21" s="9"/>
-      <x:c r="H21" s="9"/>
-    </x:row>
-    <x:row r="22" ht="22" customHeight="1">
-      <x:c r="A22" s="9"/>
-      <x:c r="B22" s="9"/>
-      <x:c r="C22" s="9"/>
-      <x:c r="D22" s="9"/>
-      <x:c r="E22" s="9"/>
-      <x:c r="F22" s="9"/>
-      <x:c r="G22" s="9"/>
-      <x:c r="H22" s="9"/>
-    </x:row>
-    <x:row r="23" ht="22" customHeight="1">
-      <x:c r="A23" s="9"/>
-      <x:c r="B23" s="9"/>
-      <x:c r="C23" s="9"/>
-      <x:c r="D23" s="9"/>
-      <x:c r="E23" s="9"/>
-      <x:c r="F23" s="9"/>
-      <x:c r="G23" s="9"/>
-      <x:c r="H23" s="9"/>
-    </x:row>
-    <x:row r="24" ht="22" customHeight="1">
-      <x:c r="A24" s="9"/>
-      <x:c r="B24" s="9"/>
-      <x:c r="C24" s="9"/>
-      <x:c r="D24" s="9"/>
-      <x:c r="E24" s="9"/>
-      <x:c r="F24" s="9"/>
-      <x:c r="G24" s="9"/>
-      <x:c r="H24" s="9"/>
-    </x:row>
-    <x:row r="25" ht="22" customHeight="1">
-      <x:c r="A25" s="9"/>
-      <x:c r="B25" s="9"/>
-      <x:c r="C25" s="9"/>
-      <x:c r="D25" s="9"/>
-      <x:c r="E25" s="9"/>
-      <x:c r="F25" s="9"/>
-      <x:c r="G25" s="9"/>
-      <x:c r="H25" s="9"/>
-    </x:row>
-    <x:row r="26" ht="22" customHeight="1">
-      <x:c r="A26" s="9"/>
-      <x:c r="B26" s="9"/>
-      <x:c r="C26" s="9"/>
-      <x:c r="D26" s="9"/>
-      <x:c r="E26" s="9"/>
-      <x:c r="F26" s="9"/>
-      <x:c r="G26" s="9"/>
-      <x:c r="H26" s="9"/>
-    </x:row>
-    <x:row r="27" ht="22" customHeight="1">
-      <x:c r="A27" s="9"/>
-      <x:c r="B27" s="9"/>
-      <x:c r="C27" s="9"/>
-      <x:c r="D27" s="9"/>
-      <x:c r="E27" s="9"/>
-      <x:c r="F27" s="9"/>
-      <x:c r="G27" s="9"/>
-      <x:c r="H27" s="9"/>
-    </x:row>
-    <x:row r="28" ht="22" customHeight="1">
-      <x:c r="A28" s="9"/>
-      <x:c r="B28" s="9"/>
-      <x:c r="C28" s="9"/>
-      <x:c r="D28" s="9"/>
-      <x:c r="E28" s="9"/>
-      <x:c r="F28" s="9"/>
-      <x:c r="G28" s="9"/>
-      <x:c r="H28" s="9"/>
-    </x:row>
-    <x:row r="29" ht="22" customHeight="1">
-      <x:c r="A29" s="9"/>
-      <x:c r="B29" s="9"/>
-      <x:c r="C29" s="9"/>
-      <x:c r="D29" s="9"/>
-      <x:c r="E29" s="9"/>
-      <x:c r="F29" s="9"/>
-      <x:c r="G29" s="9"/>
-      <x:c r="H29" s="9"/>
-    </x:row>
-    <x:row r="30" ht="22" customHeight="1">
-      <x:c r="A30" s="9"/>
-      <x:c r="B30" s="9"/>
-      <x:c r="C30" s="9"/>
-      <x:c r="D30" s="9"/>
-      <x:c r="E30" s="9"/>
-      <x:c r="F30" s="9"/>
-      <x:c r="G30" s="9"/>
-      <x:c r="H30" s="9"/>
-    </x:row>
-    <x:row r="31" ht="22" customHeight="1">
-      <x:c r="A31" s="9"/>
-      <x:c r="B31" s="9"/>
-      <x:c r="C31" s="9"/>
-      <x:c r="D31" s="9"/>
-      <x:c r="E31" s="9"/>
-      <x:c r="F31" s="9"/>
-      <x:c r="G31" s="9"/>
-      <x:c r="H31" s="9"/>
-    </x:row>
-    <x:row r="32" ht="22" customHeight="1">
-      <x:c r="A32" s="9"/>
-      <x:c r="B32" s="9"/>
-      <x:c r="C32" s="9"/>
-      <x:c r="D32" s="9"/>
-      <x:c r="E32" s="9"/>
-      <x:c r="F32" s="9"/>
-      <x:c r="G32" s="9"/>
-      <x:c r="H32" s="9"/>
-    </x:row>
-    <x:row r="33" ht="22" customHeight="1">
-      <x:c r="A33" s="9"/>
-      <x:c r="B33" s="9"/>
-      <x:c r="C33" s="9"/>
-      <x:c r="D33" s="9"/>
-      <x:c r="E33" s="9"/>
-      <x:c r="F33" s="9"/>
-      <x:c r="G33" s="9"/>
-      <x:c r="H33" s="9"/>
-    </x:row>
-    <x:row r="34" ht="22" customHeight="1">
-      <x:c r="A34" s="9"/>
-      <x:c r="B34" s="9"/>
-      <x:c r="C34" s="9"/>
-      <x:c r="D34" s="9"/>
-      <x:c r="E34" s="9"/>
-      <x:c r="F34" s="9"/>
-      <x:c r="G34" s="9"/>
-      <x:c r="H34" s="9"/>
-    </x:row>
-    <x:row r="35" ht="22" customHeight="1">
-      <x:c r="A35" s="9"/>
-      <x:c r="B35" s="9"/>
-      <x:c r="C35" s="9"/>
-      <x:c r="D35" s="9"/>
-      <x:c r="E35" s="9"/>
-      <x:c r="F35" s="9"/>
-      <x:c r="G35" s="9"/>
-      <x:c r="H35" s="9"/>
-    </x:row>
-    <x:row r="36" ht="22" customHeight="1">
-      <x:c r="A36" s="9"/>
-      <x:c r="B36" s="9"/>
-      <x:c r="C36" s="9"/>
-      <x:c r="D36" s="9"/>
-      <x:c r="E36" s="9"/>
-      <x:c r="F36" s="9"/>
-      <x:c r="G36" s="9"/>
-      <x:c r="H36" s="9"/>
-    </x:row>
-    <x:row r="37" ht="22" customHeight="1">
-      <x:c r="A37" s="9"/>
-      <x:c r="B37" s="9"/>
-      <x:c r="C37" s="9"/>
-      <x:c r="D37" s="9"/>
-      <x:c r="E37" s="9"/>
-      <x:c r="F37" s="9"/>
-      <x:c r="G37" s="9"/>
-      <x:c r="H37" s="9"/>
-    </x:row>
-    <x:row r="38" ht="22" customHeight="1">
-      <x:c r="A38" s="9"/>
-      <x:c r="B38" s="9"/>
-      <x:c r="C38" s="9"/>
-      <x:c r="D38" s="9"/>
-      <x:c r="E38" s="9"/>
-      <x:c r="F38" s="9"/>
-      <x:c r="G38" s="9"/>
-      <x:c r="H38" s="9"/>
-    </x:row>
-    <x:row r="39" ht="22" customHeight="1">
-      <x:c r="A39" s="9"/>
-      <x:c r="B39" s="9"/>
-      <x:c r="C39" s="9"/>
-      <x:c r="D39" s="9"/>
-      <x:c r="E39" s="9"/>
-      <x:c r="F39" s="9"/>
-      <x:c r="G39" s="9"/>
-      <x:c r="H39" s="9"/>
-    </x:row>
-    <x:row r="40" ht="22" customHeight="1">
-      <x:c r="A40" s="9"/>
-      <x:c r="B40" s="9"/>
-      <x:c r="C40" s="9"/>
-      <x:c r="D40" s="9"/>
-      <x:c r="E40" s="9"/>
-      <x:c r="F40" s="9"/>
-      <x:c r="G40" s="9"/>
-      <x:c r="H40" s="9"/>
-    </x:row>
-    <x:row r="41" ht="22" customHeight="1">
-      <x:c r="A41" s="9"/>
-      <x:c r="B41" s="9"/>
-      <x:c r="C41" s="9"/>
-      <x:c r="D41" s="9"/>
-      <x:c r="E41" s="9"/>
-      <x:c r="F41" s="9"/>
-      <x:c r="G41" s="9"/>
-      <x:c r="H41" s="9"/>
-    </x:row>
-    <x:row r="42" ht="22" customHeight="1">
-      <x:c r="A42" s="9"/>
-      <x:c r="B42" s="9"/>
-      <x:c r="C42" s="9"/>
-      <x:c r="D42" s="9"/>
-      <x:c r="E42" s="9"/>
-      <x:c r="F42" s="9"/>
-      <x:c r="G42" s="9"/>
-      <x:c r="H42" s="9"/>
-    </x:row>
-    <x:row r="43" ht="22" customHeight="1">
-      <x:c r="A43" s="9"/>
-      <x:c r="B43" s="9"/>
-      <x:c r="C43" s="9"/>
-      <x:c r="D43" s="9"/>
-      <x:c r="E43" s="9"/>
-      <x:c r="F43" s="9"/>
-      <x:c r="G43" s="9"/>
-      <x:c r="H43" s="9"/>
-    </x:row>
-    <x:row r="44" ht="22" customHeight="1">
-      <x:c r="A44" s="9"/>
-      <x:c r="B44" s="9"/>
-      <x:c r="C44" s="9"/>
-      <x:c r="D44" s="9"/>
-      <x:c r="E44" s="9"/>
-      <x:c r="F44" s="9"/>
-      <x:c r="G44" s="9"/>
-      <x:c r="H44" s="9"/>
-    </x:row>
-    <x:row r="45" ht="22" customHeight="1">
-      <x:c r="A45" s="9"/>
-      <x:c r="B45" s="9"/>
-      <x:c r="C45" s="9"/>
-      <x:c r="D45" s="9"/>
-      <x:c r="E45" s="9"/>
-      <x:c r="F45" s="9"/>
-      <x:c r="G45" s="9"/>
-      <x:c r="H45" s="9"/>
-    </x:row>
-    <x:row r="46" ht="22" customHeight="1">
-      <x:c r="A46" s="9"/>
-      <x:c r="B46" s="9"/>
-      <x:c r="C46" s="9"/>
-      <x:c r="D46" s="9"/>
-      <x:c r="E46" s="9"/>
-      <x:c r="F46" s="9"/>
-      <x:c r="G46" s="9"/>
-      <x:c r="H46" s="9"/>
-    </x:row>
-    <x:row r="47" ht="22" customHeight="1">
-      <x:c r="A47" s="9"/>
-      <x:c r="B47" s="9"/>
-      <x:c r="C47" s="9"/>
-      <x:c r="D47" s="9"/>
-      <x:c r="E47" s="9"/>
-      <x:c r="F47" s="9"/>
-      <x:c r="G47" s="9"/>
-      <x:c r="H47" s="9"/>
-    </x:row>
-    <x:row r="48" ht="22" customHeight="1">
-      <x:c r="A48" s="9"/>
-      <x:c r="B48" s="9"/>
-      <x:c r="C48" s="9"/>
-      <x:c r="D48" s="9"/>
-      <x:c r="E48" s="9"/>
-      <x:c r="F48" s="9"/>
-      <x:c r="G48" s="9"/>
-      <x:c r="H48" s="9"/>
-    </x:row>
-    <x:row r="49" ht="22" customHeight="1">
-      <x:c r="A49" s="9"/>
-      <x:c r="B49" s="9"/>
-      <x:c r="C49" s="9"/>
-      <x:c r="D49" s="9"/>
-      <x:c r="E49" s="9"/>
-      <x:c r="F49" s="9"/>
-      <x:c r="G49" s="9"/>
-      <x:c r="H49" s="9"/>
-    </x:row>
-    <x:row r="50" ht="22" customHeight="1">
-      <x:c r="A50" s="9"/>
-      <x:c r="B50" s="9"/>
-      <x:c r="C50" s="9"/>
-      <x:c r="D50" s="9"/>
-      <x:c r="E50" s="9"/>
-      <x:c r="F50" s="9"/>
-      <x:c r="G50" s="9"/>
-      <x:c r="H50" s="9"/>
-    </x:row>
-    <x:row r="51" ht="22" customHeight="1">
-      <x:c r="A51" s="9"/>
-      <x:c r="B51" s="9"/>
-      <x:c r="C51" s="9"/>
-      <x:c r="D51" s="9"/>
-      <x:c r="E51" s="9"/>
-      <x:c r="F51" s="9"/>
-      <x:c r="G51" s="9"/>
-      <x:c r="H51" s="9"/>
+    <x:row r="2" ht="28" customHeight="1">
+      <x:c r="A2" s="9" t="n">
+        <x:v>11.45</x:v>
+      </x:c>
+      <x:c r="B2" s="7" t="str">
+        <x:v>1D36间距200</x:v>
+      </x:c>
+      <x:c r="C2" s="7" t="str">
+        <x:v>1D40间距200</x:v>
+      </x:c>
+      <x:c r="D2" s="8"/>
+      <x:c r="E2" s="8"/>
+      <x:c r="F2" s="7" t="str">
+        <x:v>1D36间距200</x:v>
+      </x:c>
+      <x:c r="G2" s="7" t="str">
+        <x:v>1D40间距200</x:v>
+      </x:c>
+      <x:c r="H2" s="7" t="str">
+        <x:v>1D16间距200</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>